<commit_message>
update wordalsiation + fex shot
</commit_message>
<xml_diff>
--- a/data/describe/few_shot/cluster/messages_country.xlsx
+++ b/data/describe/few_shot/cluster/messages_country.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x15 xr xr6 xr10">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\amaca253\Documents\datomatisation\datomatisation-dev\data\describe\few_shot\cluster\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:40009_{29CA6663-2A3C-43D0-ADCC-15DE01478D04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6851E3FB-13A9-4012-9E79-A94B659AB57D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="53295" yWindow="2640" windowWidth="23370" windowHeight="16800"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="QandA_data" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
   <si>
     <t>User</t>
   </si>
@@ -33,139 +33,61 @@
     <t>Assistant</t>
   </si>
   <si>
-    <t>What does it mean when a country is described as confident and engaged?</t>
-  </si>
-  <si>
-    <t>When a country is described as confident and engaged, it showcases a spirit of active participation and trust among its citizens. People are likely to view political engagement, like signing electronic petitions, as a positive action, and they tend to have a strong belief in the importance of faith, while also trusting others, including those from different nationalities. This creates a vibrant atmosphere where individuals feel empowered and connected to one another and their governance.</t>
-  </si>
-  <si>
-    <t>What does it mean when a country is described as concerned and cautious?</t>
-  </si>
-  <si>
-    <t>When a country is described as concerned and cautious, it indicates a deep sense of worry about various critical issues. This includes significant fears about providing quality education for future generations, anxieties over potential civil conflict and war, and worries about job security and employment prospects. Overall, such a country tends to approach situations with a careful and apprehensive mindset, reflecting a desire to protect its citizens from uncertainty and challenges.</t>
-  </si>
-  <si>
-    <t>What does it mean when a country is described as principled?</t>
-  </si>
-  <si>
-    <t>When a country is described as principled, it indicates that there is a measured level of confidence in its political structures, such as political parties, parliament, and government, even if that confidence is not overwhelmingly high. This suggests that the country values integrity and has a sense of ethical responsibility in its governance, contrasting sharply with a lack of concern for moral standards.</t>
-  </si>
-  <si>
-    <t>What does it mean when a country is described as indifferent?</t>
-  </si>
-  <si>
-    <t>When a country is described as indifferent, it means that there is a troubling ease with which certain behaviors, such as stealing, violence, accepting bribes, domestic abuse, and tax cheating, can be justified. This reflects a lack of ethical conviction where right and wrong become blurred, indicating a society that may turn a blind eye to moral transgressions.</t>
-  </si>
-  <si>
-    <t>What does it mean when a country is described as active and involved?</t>
-  </si>
-  <si>
-    <t>When a country is described as active and involved, it means that its citizens actively participate in various organizations, such as charitable or professional groups, showing a strong commitment to community engagement. This enthusiasm extends to support for self-help or consumer organizations, highlighting a vibrant participation that fosters connections and collective action.</t>
-  </si>
-  <si>
-    <t>What does it mean when a country is described as passive and distant?</t>
-  </si>
-  <si>
-    <t>When a country is described as passive and distant, it suggests a lack of engagement and reluctance to take action on significant issues. People in such a country may be less likely to participate in petitions or political actions, exhibit a general distrust towards those of different backgrounds, and report feelings of unhappiness, reflecting a disengaged and aloof society.</t>
-  </si>
-  <si>
-    <t>What does it mean when a country is described as trusted?</t>
-  </si>
-  <si>
-    <t>When a country is described as trusted, it indicates a strong sense of confidence that its government, parliament, political parties, civil services, and justice system can be relied upon. This trust reflects a belief that these institutions operate effectively and with integrity, fostering a sense of security and assurance among the citizens.</t>
+    <t>What does it mean when a country is described as unconfident?</t>
+  </si>
+  <si>
+    <t>When a country is described as unconfident, it reflects a sense of hesitancy or doubt about its political institutions, such as a weak confidence in political parties and parliament. This feeling extends to social values, where there might be uncertainty about the implications of prioritizing personal well-being over work, indicating a lack of assurance in the nationâ€™s collective direction and decisions.</t>
+  </si>
+  <si>
+    <t>What does it mean when a country is described as justifiable?</t>
+  </si>
+  <si>
+    <t>When a country is described as justifiable, it reflects a perspective where actions like stealing property, violence against others, accepting bribes, domestic abuse, and cheating on taxes are viewed through a lens of acceptability, suggesting that there are situations where these behaviors might seem reasonable or warranted. This stance encompasses a belief system that frequently justifies morally questionable actions, contributing to a broader understanding of social norms and ethics within that country.</t>
+  </si>
+  <si>
+    <t>What does it mean when a country is described as trusting?</t>
+  </si>
+  <si>
+    <t>When a country is described as trusting, it reflects a belief that most people can be relied upon and that there is a strong sense of confidence in both personal relationships and those across national boundaries. This trust extends beyond just individuals, highlighting the importance of faith in God and an openness to engage in political actions, such as signing electronic petitions, indicating a society that values cooperation and connection.</t>
+  </si>
+  <si>
+    <t>What does it mean when a country is described as concerned?</t>
+  </si>
+  <si>
+    <t>When a country is described as concerned, it means that its citizens are deeply troubled by various social issues and potential threats. They worry significantly about matters like education for future generations, the justifiability of abortion and homosexuality, and even the looming fear of civil unrest, indicating a collective anxiety about the moral and societal direction of their nation.</t>
+  </si>
+  <si>
+    <t>What does it mean when a country is described as confident?</t>
+  </si>
+  <si>
+    <t>When a country is described as confident, it means that its citizens have a strong trust in their government, parliament, and civil service, feeling secure in the systems that govern their lives. This confidence extends notably to their justice system and political parties, suggesting a robust belief in the overall integrity and effectiveness of their institutions.</t>
   </si>
   <si>
     <t>What does it mean when a country is described as skeptical?</t>
   </si>
   <si>
-    <t>When a country is described as skeptical, it reflects a general uncertainty about traditional authority and the importance placed on obedience, respect, and leisure time. This means that residents may question whether greater respect for authority is a positive step, showcasing a cautious outlook towards established power structures and values in society.</t>
-  </si>
-  <si>
-    <t>What does it mean when a country is described as involved and committed?</t>
-  </si>
-  <si>
-    <t>When a country is described as involved and committed, it reflects a community where citizens actively participate in various organizations, from professional and consumer groups to charitable and self-help initiatives. Additionally, thereâ€™s a sense of personal significance placed on beliefs and values, highlighting a connection to the role of faith in their lives. This involvement indicates a vibrant social fabric, where individuals care about their contributions and the welfare of their society.</t>
-  </si>
-  <si>
-    <t>What does it mean when a country is described as disengaged and indifferent?</t>
-  </si>
-  <si>
-    <t>When a country is described as disengaged and indifferent, it reflects a lack of connection and commitment to community and societal values. Citizens may not prioritize instilling religious faith in children, feel little pride in their nationality, and show skepticism towards the role of work in contributing to society, leading to an overall sense of disinterest and detachment from important aspects of a shared national identity.</t>
-  </si>
-  <si>
-    <t>What does it mean when a country is described as unworried?</t>
-  </si>
-  <si>
-    <t>When a country is described as unworried, it means that the nation does not have significant concerns about various threats, such as terrorist attacks, war, or civil unrest. In essence, this country exhibits a sense of calmness, free from the anxieties that might plague others regarding safety and security.</t>
-  </si>
-  <si>
-    <t>What does it mean when a country is described as anxious and fearful?</t>
-  </si>
-  <si>
-    <t>When a country is described as anxious and fearful, it reflects a sense of unease and concern about potential threats. Citizens may express worries about serious issues, such as the possibility of a terrorist attack, an impending war, or even a civil war, indicating that there is a prevailing atmosphere of apprehension and dread within the nation.</t>
-  </si>
-  <si>
-    <t>What does it mean when a country is described as participative and engaged?</t>
-  </si>
-  <si>
-    <t>When a country is described as participative and engaged, it means that its citizens tend to be involved in various organizations, such as professional and charitable groups, showing a willingness to contribute to society. Additionally, they value the importance of passing on religious beliefs to the next generation, reflecting an active engagement in both community and family values.</t>
-  </si>
-  <si>
-    <t>What does it mean when a country is described as not participative?</t>
-  </si>
-  <si>
-    <t>When a country is described as not participative, it suggests a lack of involvement in organizations and community activities. Citizens are not actively engaging in professional, charitable, or even spiritual realms, indicating a general disinterest in collaborative efforts and civic responsibility.</t>
-  </si>
-  <si>
-    <t>What does it mean when a country is described as satisfied and secure?</t>
-  </si>
-  <si>
-    <t>When a country is described as satisfied and secure, it reflects a sense of contentment and stability among its people. This can be seen in moderate life satisfaction levels, where individuals generally feel pleased with their lives, alongside a general trust in their neighborhoods and families, indicating a community that feels united and dependable.</t>
-  </si>
-  <si>
-    <t>What does it mean when a country is described as uncertain and hesitant?</t>
-  </si>
-  <si>
-    <t>When a country is described as uncertain and hesitant, it reflects a state of indecision and doubt about its overall happiness and contentment. This uncertainty suggests that citizens may struggle to feel truly joyful or confident in their circumstances, presenting a landscape where satisfaction is elusive.</t>
-  </si>
-  <si>
-    <t>What does it mean when a country is described as trusting?</t>
-  </si>
-  <si>
-    <t>When a country is described as trusting, it reflects a general belief in the goodness of others, as seen in the way its citizens feel secure in their neighborhoods and are open to trusting people from different religions and nationalities. This sense of trust also extends to new acquaintances, suggesting a welcoming spirit and confidence in relationships with others.</t>
-  </si>
-  <si>
-    <t>What does it mean when a country is described as mistrusting?</t>
-  </si>
-  <si>
-    <t>When a country is described as mistrusting, it means that its people tend to not trust others easily, whether it involves new acquaintances, those from different religions, or individuals of varying nationalities. This lack of trust can create an atmosphere of skepticism and uncertainty, where people are cautious and hesitant to engage with others fully.</t>
-  </si>
-  <si>
-    <t>This cluster characterizes countries that display a general sense of disengagement and anxiety in their societal dynamics. Despite being principled and maintaining a degree of participation, these countries struggle with lower levels of trust and satisfaction, suggesting a community that is not fully confident in its engagement. The notable weaknesses in this cluster lie in their high levels of anxiety and fearfulness, combined with a tendency towards disengagement and indifference, which may hinder progress and collaboration among their citizens.</t>
-  </si>
-  <si>
-    <t>This cluster represents countries that exhibit a reserved approach towards engagement and commitment, characterized by a noticeable lack of confidence and proactivity. Specific strengths include a principled stance on issues and a stable score on participative engagement, suggesting a balanced approach to civic involvement when prompted. However, the cluster faces weaknesses in its skepticism, low levels of active participation, and a tendency toward uncertainty, which may hinder effective collaboration and positive progress on relevant social issues.</t>
-  </si>
-  <si>
-    <t>This cluster represents countries characterized by a cautious and somewhat disengaged demeanor. The members of this cluster display a notable strength in their awareness of potential risks, as indicated by their high levels of concern and skepticism, alongside a pronounced anxiety about their circumstances. However, their specific weaknesses lie in their low levels of trust and participation, which may hinder their ability to effectively address challenges and foster a sense of community engagement.</t>
-  </si>
-  <si>
-    <t>This cluster represents a group characterized by a tendency towards disengagement and distance. Members exhibit a notable level of caution and trust, but their hesitance and passivity indicate a lack of proactive involvement in various matters. The primary weakness of this cluster lies in its high levels of uncertainty and disengagement, which may hinder effective collaboration and responsiveness in dynamic environments.</t>
-  </si>
-  <si>
-    <t>This cluster consists of countries that display a notable degree of concern and caution, reflecting a reserved approach to engagement. The strengths of this cluster include a structured perspective that often results in careful deliberation on issues, though this cautiousness may also foster a sense of indifference in their response to various initiatives. However, the specific weaknesses of this cluster lie in their low levels of participation and trust, indicating a potential challenge in fostering committed and collaborative relationships both domestically and internationally.</t>
-  </si>
-  <si>
-    <t>This cluster represents a group of countries showcasing a significant level of indifference and skepticism, reflecting a low commitment to civic engagement. Their specific strengths lie in a high degree of passive observation and express skepticism about participatory initiatives, highlighting a tendency to critically assess their environments. However, this cluster faces notable weaknesses, such as low levels of satisfaction and security, an overwhelming sense of mistrust, and a disengaged outlook that may hinder social cohesion and progress.</t>
-  </si>
-  <si>
-    <t>Members of this cluster exhibit a predominant tendency towards concern and caution, suggesting a heightened sensitivity to risks and uncertainties. Their skepticism and disengagement may reflect a lack of active involvement in societal matters, paired with a significant mistrust in external systems or institutions. However, this cluster also shows vulnerabilities, particularly in their lower levels of satisfaction and security, which may hinder their overall confidence and engagement in various aspects of life.</t>
-  </si>
-  <si>
-    <t>This cluster represents countries characterized by a significant lack of confidence and engagement, which results in a cautious and hesitant outlook. A specific strength of this cluster is that while they are reasonably trusted, they struggle with high levels of uncertainty and mistrust towards other entities. The notable weakness lies in their very low levels of participation and commitment, coupled with a marked tendency to remain passive and distant, leading to challenges in fostering proactive governance and societal involvement.</t>
-  </si>
-  <si>
-    <t>This cluster depicts a group characterized by a generally cautious approach, coupled with a slight tendency towards skepticism and passivity. Their notable strengths lie in their satisfaction and security, alongside a balanced outlook, implying some stability in their perspective. However, the cluster struggles with low levels of principled actions, involvement, and trust, which may hinder their progress and engagement with broader societal issues.</t>
+    <t>When a country is described as skeptical, it conveys a sense of hesitation or doubt regarding certain activities and beliefs. This skepticism is reflected in the lower importance placed on leisure time and a reluctance toward participating in actions like signing petitions, suggesting a general caution or disbelief in the effectiveness or value of such engagements.</t>
+  </si>
+  <si>
+    <t>What does it mean when a country is described as active?</t>
+  </si>
+  <si>
+    <t>When a country is described as active, it means that its citizens are significantly engaged in professional, charitable, and consumer organizations, showing a commitment to community and collaboration. This vibrant participation reflects a society that values involvement and cooperation, often leading to a diverse range of initiatives that enhance social ties and support among individuals.</t>
+  </si>
+  <si>
+    <t>What does it mean when a country is described as passive?</t>
+  </si>
+  <si>
+    <t>When a country is described as passive, it suggests a tendency to shy away from active participation in political engagement, such as signing electronic petitions or taking community initiatives. This passivity reflects a reluctance to engage in actions that drive societal change, indicating a more subdued presence in active civic life.</t>
+  </si>
+  <si>
+    <t>This cluster represents countries that exhibit a balanced outlook, characterized by their normal stance on justifiability and a heightened sense of concern. Their strength lies in their ability to recognize and address pressing issues, reflecting a commitment to societal well-being. However, the cluster tends to exhibit a lack of confidence, which may hinder their proactive engagement and decision-making in challenging situations.</t>
+  </si>
+  <si>
+    <t>This cluster comprises countries that exhibit a cautious and analytical approach to situations, marked by a slight inclination towards justifiable actions. Their strengths lie in their ability to critically evaluate circumstances, which is enhanced by their high levels of skepticism, potentially leading to more robust decision-making. However, this cluster's weaknesses emerge from lower levels of trust and passivity, which might hinder collaboration and responsiveness to opportunities presented in their environment.</t>
+  </si>
+  <si>
+    <t>This cluster comprises countries that display a cautious and somewhat reserved disposition in their international and domestic interactions. Their specific strengths include a normal level of activity, suggesting they engage in various initiatives and projects, albeit with a hesitance stemming from their lower confidence levels. However, the cluster's weaknesses lie in their low levels of trust and confidence, which may hinder collaborative efforts and foster a sense of skepticism in crucial partnerships.</t>
   </si>
   <si>
     <t>Thats really good. You truly understand the factors and names. 
@@ -176,37 +98,27 @@
 The second sentence should describe the cluster’s specific strengths based on the available information.
 The third sentence should highlight areas where the cluster has specific weaknesses based on the available information.
 I will provided you with the cluster description and you will return the summary. 
-Here is the cluster description based on the factor scores at the cluster center, representing a typical country in that cluster: ```Members of this cluster can be described as:  relatively low on confident and engaged,  normal on principled,  normal on passive and distant,  relatively low on trusted,  relatively high on disengaged and indifferent,  relatively high on anxious and fearful,  normal on participative and engaged,  relatively low on satisfied and secure,  normal on mistrusting´´´</t>
-  </si>
-  <si>
-    <t>Here is the cluster description based on the factor scores at the cluster center, representing a typical country in that cluster: ```Members of this cluster can be described as: quite low on confident and engaged, normal on principled, relatively low on active and involved, relatively high on skeptical, relatively low on involved and committed, slightly low on unworried, normal on participative and engaged, normal on uncertain and hesitant, normal on trusting´´´</t>
-  </si>
-  <si>
-    <t>Here is the cluster description based on the factor scores at the cluster center, representing a typical country in that cluster: ```Members of this cluster can be described as: relatively high on concerned and cautious, relatively high on indifferent, slightly high on passive and distant, relatively high on skeptical, normal on involved and committed, very high on anxious and fearful, slightly low on participative and engaged, quite high on uncertain and hesitant, relatively low on trusting´´´</t>
-  </si>
-  <si>
-    <t>Here is the cluster description based on the factor scores at the cluster center, representing a typical country in that cluster: ```Members of this cluster can be described as:  normal on concerned and cautious,  normal on indifferent,  relatively high on passive and distant,  normal on trusted,  relatively high on disengaged and indifferent,  relatively low on unworried,  relatively low on participative and engaged,  relatively high on uncertain and hesitant,  slightly low on trusting´´´</t>
-  </si>
-  <si>
-    <t>Here is the cluster description based on the factor scores at the cluster center, representing a typical country in that cluster: ```Members of this cluster can be described as:  relatively high on concerned and cautious,  quite high on indifferent,  quite low on active and involved,  relatively low on trusted,  relatively low on involved and committed,  relatively low on unworried,  relatively high on not participative,  normal on uncertain and hesitant,  relatively low on trusting´´´</t>
-  </si>
-  <si>
-    <t>Here is the cluster description based on the factor scores at the cluster center, representing a typical country in that cluster: ```Members of this cluster can be described as:  quite low on confident and engaged,  extremely high on indifferent,  relatively high on passive and distant,  very high on skeptical,  relatively high on disengaged and indifferent,  relatively low on unworried,  normal on not participative,  very low on satisfied and secure,  very high on mistrusting´´´</t>
-  </si>
-  <si>
-    <t>Here is the cluster description based on the factor scores at the cluster center, representing a typical country in that cluster: ```Members of this cluster can be described as:  quite high on concerned and cautious,  relatively low on principled,  relatively low on active and involved,  normal on skeptical,  slightly high on disengaged and indifferent,  normal on unworried,  normal on participative and engaged,  slightly low on satisfied and secure,  quite high on mistrusting´´´</t>
-  </si>
-  <si>
-    <t>Here is the cluster description based on the factor scores at the cluster center, representing a typical country in that cluster: ```Members of this cluster can be described as:  relatively low on confident and engaged,  quite low on principled,  slightly high on passive and distant,  normal on trusted,  very low on involved and committed,  normal on anxious and fearful,  relatively low on participative and engaged,  very high on uncertain and hesitant,  extremely high on mistrusting´´´</t>
-  </si>
-  <si>
-    <t>Here is the cluster description based on the factor scores at the cluster center, representing a typical country in that cluster: ```Members of this cluster can be described as:  normal on concerned and cautious,  relatively low on principled,  slightly high on passive and distant,  slightly high on skeptical,  slightly low on involved and committed,  normal on anxious and fearful,  quite high on not participative,  normal on satisfied and secure,  relatively low on trusting´´´</t>
+Here is the cluster description based on the factor scores at the cluster center, representing a typical country in that cluster: ```Members of this cluster can be described as:  normal on justifiable,  quite high on concerned,  slightly low on confident,  normal on passive´´´</t>
+  </si>
+  <si>
+    <t>Here is the cluster description based on the factor scores at the cluster center, representing a typical country in that cluster: ```Members of this cluster can be described as:  slightly high on justifiable,  slightly low on trusting,  quite high on skeptical,  normal on passive´´´</t>
+  </si>
+  <si>
+    <t>Those were really good. Exactly what I am looking for. 
+Make sure you continue to use the same format and style in the next example. 
+I am now going to give you one last description task to complete. 
+You will receive information about the cluster based on the latent factors that best describe it.
+For each cluster, write a concise summary based on the available information.
+The first sentence should give an overview of the cluster. 
+The second sentence should describe the cluster’s specific strengths based on the available information.
+The third sentence should highlight areas where the cluster has specific weaknesses based on the available information.
+Now do the same thing with the following, here is the cluster description based on the factor scores at the cluster center, representing a typical country in that cluster: ```Members of this cluster can be described as:  slightly low on unconfident,  relatively low on trusting,  relatively low on confident,  normal on active´´´</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -343,7 +255,7 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="8"/>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -697,16 +609,13 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="42">
@@ -1062,236 +971,108 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B28"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:B12"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="88.54296875" customWidth="1"/>
-    <col min="2" max="2" width="103.7265625" customWidth="1"/>
+    <col min="1" max="1" width="70.81640625" customWidth="1"/>
+    <col min="2" max="2" width="89.81640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="52.5" x14ac:dyDescent="0.35">
-      <c r="A2" s="2" t="s">
+    <row r="2" spans="1:2" ht="52" x14ac:dyDescent="0.35">
+      <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="52.5" x14ac:dyDescent="0.35">
-      <c r="A3" s="2" t="s">
+    <row r="3" spans="1:2" ht="65" x14ac:dyDescent="0.35">
+      <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="42" x14ac:dyDescent="0.35">
-      <c r="A4" s="2" t="s">
+    <row r="4" spans="1:2" ht="52" x14ac:dyDescent="0.35">
+      <c r="A4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="42" x14ac:dyDescent="0.35">
-      <c r="A5" s="2" t="s">
+    <row r="5" spans="1:2" ht="52" x14ac:dyDescent="0.35">
+      <c r="A5" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="42" x14ac:dyDescent="0.35">
-      <c r="A6" s="2" t="s">
+    <row r="6" spans="1:2" ht="52" x14ac:dyDescent="0.35">
+      <c r="A6" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="42" x14ac:dyDescent="0.35">
-      <c r="A7" s="2" t="s">
+    <row r="7" spans="1:2" ht="52" x14ac:dyDescent="0.35">
+      <c r="A7" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="31.5" x14ac:dyDescent="0.35">
-      <c r="A8" s="2" t="s">
+    <row r="8" spans="1:2" ht="52" x14ac:dyDescent="0.35">
+      <c r="A8" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="42" x14ac:dyDescent="0.35">
-      <c r="A9" s="2" t="s">
+    <row r="9" spans="1:2" ht="39" x14ac:dyDescent="0.35">
+      <c r="A9" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:2" ht="52.5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:2" ht="130" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B10" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B10" s="2" t="s">
+    </row>
+    <row r="11" spans="1:2" ht="40" x14ac:dyDescent="0.35">
+      <c r="A11" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B11" s="2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="42" x14ac:dyDescent="0.35">
-      <c r="A11" s="2" t="s">
+    <row r="12" spans="1:2" ht="120" x14ac:dyDescent="0.35">
+      <c r="A12" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B12" s="2" t="s">
         <v>20</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" ht="31.5" x14ac:dyDescent="0.35">
-      <c r="A12" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" ht="42" x14ac:dyDescent="0.35">
-      <c r="A13" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" ht="42" x14ac:dyDescent="0.35">
-      <c r="A14" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" ht="31.5" x14ac:dyDescent="0.35">
-      <c r="A15" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" ht="42" x14ac:dyDescent="0.35">
-      <c r="A16" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" ht="31.5" x14ac:dyDescent="0.35">
-      <c r="A17" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" ht="42" x14ac:dyDescent="0.35">
-      <c r="A18" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" ht="31.5" x14ac:dyDescent="0.35">
-      <c r="A19" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" ht="131.5" x14ac:dyDescent="0.35">
-      <c r="A20" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" ht="42" x14ac:dyDescent="0.35">
-      <c r="A21" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" ht="41.5" x14ac:dyDescent="0.35">
-      <c r="A22" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="B22" s="3" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" ht="41.5" x14ac:dyDescent="0.35">
-      <c r="A23" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="B23" s="2" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" ht="41.5" x14ac:dyDescent="0.35">
-      <c r="A24" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="B24" s="3" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" ht="42" x14ac:dyDescent="0.35">
-      <c r="A25" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="B25" s="2" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" ht="41.5" x14ac:dyDescent="0.35">
-      <c r="A26" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="B26" s="3" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" ht="42" x14ac:dyDescent="0.35">
-      <c r="A27" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="B27" s="2" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" ht="41.5" x14ac:dyDescent="0.35">
-      <c r="A28" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="B28" s="3" t="s">
-        <v>46</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update f-s and app
</commit_message>
<xml_diff>
--- a/data/describe/few_shot/cluster/messages_country.xlsx
+++ b/data/describe/few_shot/cluster/messages_country.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\amaca253\Documents\datomatisation\datomatisation-dev\data\describe\few_shot\cluster\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6851E3FB-13A9-4012-9E79-A94B659AB57D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B6D593C-532D-411A-B99A-55975B769229}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,9 +36,6 @@
     <t>What does it mean when a country is described as unconfident?</t>
   </si>
   <si>
-    <t>When a country is described as unconfident, it reflects a sense of hesitancy or doubt about its political institutions, such as a weak confidence in political parties and parliament. This feeling extends to social values, where there might be uncertainty about the implications of prioritizing personal well-being over work, indicating a lack of assurance in the nationâ€™s collective direction and decisions.</t>
-  </si>
-  <si>
     <t>What does it mean when a country is described as justifiable?</t>
   </si>
   <si>
@@ -79,15 +76,6 @@
   </si>
   <si>
     <t>When a country is described as passive, it suggests a tendency to shy away from active participation in political engagement, such as signing electronic petitions or taking community initiatives. This passivity reflects a reluctance to engage in actions that drive societal change, indicating a more subdued presence in active civic life.</t>
-  </si>
-  <si>
-    <t>This cluster represents countries that exhibit a balanced outlook, characterized by their normal stance on justifiability and a heightened sense of concern. Their strength lies in their ability to recognize and address pressing issues, reflecting a commitment to societal well-being. However, the cluster tends to exhibit a lack of confidence, which may hinder their proactive engagement and decision-making in challenging situations.</t>
-  </si>
-  <si>
-    <t>This cluster comprises countries that exhibit a cautious and analytical approach to situations, marked by a slight inclination towards justifiable actions. Their strengths lie in their ability to critically evaluate circumstances, which is enhanced by their high levels of skepticism, potentially leading to more robust decision-making. However, this cluster's weaknesses emerge from lower levels of trust and passivity, which might hinder collaboration and responsiveness to opportunities presented in their environment.</t>
-  </si>
-  <si>
-    <t>This cluster comprises countries that display a cautious and somewhat reserved disposition in their international and domestic interactions. Their specific strengths include a normal level of activity, suggesting they engage in various initiatives and projects, albeit with a hesitance stemming from their lower confidence levels. However, the cluster's weaknesses lie in their low levels of trust and confidence, which may hinder collaborative efforts and foster a sense of skepticism in crucial partnerships.</t>
   </si>
   <si>
     <t>Thats really good. You truly understand the factors and names. 
@@ -114,6 +102,18 @@
 The third sentence should highlight areas where the cluster has specific weaknesses based on the available information.
 Now do the same thing with the following, here is the cluster description based on the factor scores at the cluster center, representing a typical country in that cluster: ```Members of this cluster can be described as:  slightly low on unconfident,  relatively low on trusting,  relatively low on confident,  normal on active´´´</t>
   </si>
+  <si>
+    <t>When a country is described as unconfident, it reflects a sense of hesitancy or doubt about its political institutions, such as a weak confidence in political parties and parliament. This feeling extends to social values, where there might be uncertainty about the implications of prioritizing personal well-being over work, indicating a lack of assurance in the nation's collective direction and decisions.</t>
+  </si>
+  <si>
+    <t>They maintain a steady pulse of activity and participate in a wide range of initiatives, they do so with a hand on the brake. Their efforts are consistently tempered by a crisis of confidence. Because they lead with skepticism rather than trust, these nations often struggle to turn routine participation into the deep, high-stakes partnerships required for global impact.</t>
+  </si>
+  <si>
+    <t>Those countries that exhibit a cautious and analytical approach to situations, marked by a slight inclination towards justifiable actions. Driven by high skepticism and a demand for justification, these countries excel at making robust decisions. However, their high skepticism often breeds low trust, resulting in a passivity that can cause them to miss the window of opportunity for global collaboration.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Those countries exhibit a balanced outlook, characterized by their normal stance on justifiability and a heightened sense of concern. While they possess a sharp, balanced understanding of global issues and a deep commitment to societal well-being, they are held back by a quiet crisis of confidence. </t>
+  </si>
 </sst>
 </file>
 
@@ -262,7 +262,7 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="8"/>
+      <sz val="9"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
@@ -975,7 +975,7 @@
   <dimension ref="A1:B12"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="70.81640625" customWidth="1"/>
+    <col min="1" max="1" width="74.453125" customWidth="1"/>
     <col min="2" max="2" width="89.81640625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -992,87 +992,87 @@
         <v>2</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>3</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="65" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>4</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="52" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>6</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="52" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>8</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="52" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>10</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="52" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" s="1" t="s">
         <v>12</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="52" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" s="1" t="s">
         <v>14</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="39" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B9" s="1" t="s">
+    </row>
+    <row r="10" spans="1:2" ht="161" x14ac:dyDescent="0.35">
+      <c r="A10" s="2" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="10" spans="1:2" ht="130" x14ac:dyDescent="0.35">
-      <c r="A10" s="2" t="s">
+      <c r="B10" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="46" x14ac:dyDescent="0.35">
+      <c r="A11" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" ht="161" x14ac:dyDescent="0.35">
+      <c r="A12" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B12" s="2" t="s">
         <v>21</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" ht="40" x14ac:dyDescent="0.35">
-      <c r="A11" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" ht="120" x14ac:dyDescent="0.35">
-      <c r="A12" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>